<commit_message>
added sliding window problems
</commit_message>
<xml_diff>
--- a/documents/plan/90_Day_SDE_Daily_Tracker.xlsx
+++ b/documents/plan/90_Day_SDE_Daily_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Target-learn\documents\plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF28925-69B4-4B66-BBFB-444928934B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3606E008-A6C6-482D-B5A0-8AE983F33727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Tracker" sheetId="1" r:id="rId1"/>
@@ -1538,7 +1538,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N91"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="7" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
@@ -1554,7 +1554,7 @@
     <col min="13" max="13" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="N2" s="2"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="N3" s="2"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="N4" s="2"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="N5" s="2"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="N11" s="2"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="N14" s="2"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="N15" s="2"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="N16" s="2"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="N17" s="2"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="N18" s="2"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="N19" s="2"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="N20" s="2"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -2396,7 +2396,7 @@
       </c>
       <c r="N21" s="2"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="N22" s="2"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="N23" s="2"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="N24" s="2"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="N25" s="2"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="N28" s="2"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="N30" s="2"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="N31" s="2"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="N32" s="2"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="N33" s="2"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="N34" s="2"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="N35" s="2"/>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="N36" s="2"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="N37" s="2"/>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="N38" s="2"/>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="N39" s="2"/>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="N40" s="2"/>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="N41" s="2"/>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -3236,7 +3236,7 @@
       </c>
       <c r="N42" s="2"/>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="N43" s="2"/>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="N44" s="2"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -3356,7 +3356,7 @@
       </c>
       <c r="N45" s="2"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="N46" s="2"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="N47" s="2"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="N48" s="2"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="N49" s="2"/>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -3556,7 +3556,7 @@
       </c>
       <c r="N50" s="2"/>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="N51" s="2"/>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="N52" s="2"/>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -3676,7 +3676,7 @@
       </c>
       <c r="N53" s="2"/>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="N54" s="2"/>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -3756,7 +3756,7 @@
       </c>
       <c r="N55" s="2"/>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="N56" s="2"/>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="N57" s="2"/>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="N58" s="2"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="N59" s="2"/>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -3956,7 +3956,7 @@
       </c>
       <c r="N60" s="2"/>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="N61" s="2"/>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="N62" s="2"/>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="N63" s="2"/>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="N64" s="2"/>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="N65" s="2"/>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="N66" s="2"/>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -4236,7 +4236,7 @@
       </c>
       <c r="N67" s="2"/>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="N68" s="2"/>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -4316,7 +4316,7 @@
       </c>
       <c r="N69" s="2"/>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="N70" s="2"/>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="N71" s="2"/>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="N72" s="2"/>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -4476,7 +4476,7 @@
       </c>
       <c r="N73" s="2"/>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="N74" s="2"/>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="N75" s="2"/>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="N76" s="2"/>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -4636,7 +4636,7 @@
       </c>
       <c r="N77" s="2"/>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="N78" s="2"/>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="N79" s="2"/>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="N80" s="2"/>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="N81" s="2"/>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="N82" s="2"/>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="N83" s="2"/>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="N84" s="2"/>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="N85" s="2"/>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="N86" s="2"/>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="N87" s="2"/>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="N88" s="2"/>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="N89" s="2"/>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="N90" s="2"/>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -5218,19 +5218,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>371</v>
       </c>
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>286</v>
       </c>
@@ -5238,7 +5238,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>288</v>
       </c>
@@ -5246,7 +5246,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>289</v>
       </c>
@@ -5255,7 +5255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>290</v>
       </c>
@@ -5264,7 +5264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -5273,7 +5273,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>291</v>
       </c>
@@ -5282,7 +5282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>292</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>293</v>
       </c>
@@ -5300,7 +5300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>294</v>
       </c>
@@ -5308,7 +5308,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>295</v>
       </c>
@@ -5316,7 +5316,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>296</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>297</v>
       </c>
@@ -5332,7 +5332,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>299</v>
       </c>
@@ -5340,7 +5340,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>301</v>
       </c>
@@ -5355,8 +5355,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -5367,7 +5368,7 @@
     <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>303</v>
       </c>
@@ -5393,7 +5394,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>311</v>
       </c>
@@ -5419,7 +5420,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>311</v>
       </c>
@@ -5445,7 +5446,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>311</v>
       </c>
@@ -5471,7 +5472,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>311</v>
       </c>
@@ -5497,7 +5498,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>311</v>
       </c>
@@ -5523,7 +5524,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>311</v>
       </c>
@@ -5549,7 +5550,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>311</v>
       </c>
@@ -5575,7 +5576,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>311</v>
       </c>
@@ -5601,7 +5602,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>311</v>
       </c>
@@ -5627,7 +5628,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>311</v>
       </c>
@@ -5653,7 +5654,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>311</v>
       </c>
@@ -5679,7 +5680,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>311</v>
       </c>
@@ -5705,7 +5706,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>311</v>
       </c>
@@ -5731,7 +5732,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>327</v>
       </c>
@@ -5757,7 +5758,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>327</v>
       </c>
@@ -5783,7 +5784,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>327</v>
       </c>
@@ -5809,7 +5810,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>327</v>
       </c>
@@ -5835,7 +5836,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>327</v>
       </c>
@@ -5861,7 +5862,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>332</v>
       </c>
@@ -5887,7 +5888,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>332</v>
       </c>
@@ -5913,7 +5914,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>332</v>
       </c>
@@ -5939,7 +5940,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>336</v>
       </c>
@@ -5965,7 +5966,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>336</v>
       </c>
@@ -5991,7 +5992,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>336</v>
       </c>
@@ -6017,7 +6018,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>336</v>
       </c>
@@ -6043,7 +6044,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>341</v>
       </c>
@@ -6069,7 +6070,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>341</v>
       </c>
@@ -6095,7 +6096,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>344</v>
       </c>
@@ -6121,7 +6122,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>344</v>
       </c>
@@ -6147,7 +6148,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>344</v>
       </c>
@@ -6173,7 +6174,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>348</v>
       </c>
@@ -6199,7 +6200,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>348</v>
       </c>
@@ -6225,7 +6226,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>348</v>
       </c>
@@ -6251,7 +6252,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>348</v>
       </c>
@@ -6277,7 +6278,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>353</v>
       </c>
@@ -6303,7 +6304,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>353</v>
       </c>
@@ -6329,7 +6330,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>353</v>
       </c>
@@ -6355,7 +6356,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>357</v>
       </c>
@@ -6381,7 +6382,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>357</v>
       </c>
@@ -6407,7 +6408,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>357</v>
       </c>
@@ -6434,7 +6435,17 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H41" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:H41" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Cloud"/>
+        <filter val="CS"/>
+        <filter val="Distributed"/>
+        <filter val="HLD"/>
+        <filter val="LLD"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="2">
     <dataValidation type="list" sqref="D2:D42" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"No,Yes,Partial"</formula1>
@@ -6450,52 +6461,52 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>370</v>
       </c>

</xml_diff>